<commit_message>
ok, updated March 2025
</commit_message>
<xml_diff>
--- a/CT.xlsx
+++ b/CT.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="6" max="6" width="20.7109375" style="2" customWidth="1"/>
@@ -364,17 +364,17 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Cidade</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Ano</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Mês</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Cidade</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -396,17 +396,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Janeiro</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
         </is>
       </c>
       <c r="F2" s="2">
@@ -416,17 +416,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Fevereiro</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
         </is>
       </c>
       <c r="F3" s="2">
@@ -436,17 +436,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Março</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
         </is>
       </c>
       <c r="D4">
@@ -459,24 +459,24 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Abril</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D5">
-        <v>548.29</v>
+        <v>530.74</v>
       </c>
       <c r="E5">
-        <v>2.58</v>
+        <v>-0.7</v>
       </c>
       <c r="F5" s="2">
         <v>45017</v>
@@ -485,17 +485,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Maio</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
         </is>
       </c>
       <c r="F6" s="2">
@@ -505,21 +505,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Junho</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D7">
-        <v>567.5700000000001</v>
+        <v>560.29</v>
       </c>
       <c r="F7" s="2">
         <v>45078</v>
@@ -528,24 +528,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Julho</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D8">
-        <v>532.71</v>
+        <v>547.9400000000001</v>
       </c>
       <c r="E8">
-        <v>-6.14</v>
+        <v>-2.2</v>
       </c>
       <c r="F8" s="2">
         <v>45108</v>
@@ -554,24 +554,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D9">
-        <v>537.4</v>
+        <v>528.54</v>
       </c>
       <c r="E9">
-        <v>0.88</v>
+        <v>-3.54</v>
       </c>
       <c r="F9" s="2">
         <v>45139</v>
@@ -580,24 +580,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Setembro</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D10">
-        <v>547.47</v>
+        <v>514.08</v>
       </c>
       <c r="E10">
-        <v>1.87</v>
+        <v>-2.74</v>
       </c>
       <c r="F10" s="2">
         <v>45170</v>
@@ -606,24 +606,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Outubro</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D11">
-        <v>505.62</v>
+        <v>504.5</v>
       </c>
       <c r="E11">
-        <v>-7.64</v>
+        <v>-1.86</v>
       </c>
       <c r="F11" s="2">
         <v>45200</v>
@@ -632,24 +632,24 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Novembro</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D12">
-        <v>510.87</v>
+        <v>547.5700000000001</v>
       </c>
       <c r="E12">
-        <v>1.04</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="F12" s="2">
         <v>45231</v>
@@ -658,24 +658,24 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Dezembro</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D13">
-        <v>518.92</v>
+        <v>542.55</v>
       </c>
       <c r="E13">
-        <v>1.58</v>
+        <v>-0.92</v>
       </c>
       <c r="F13" s="2">
         <v>45261</v>
@@ -684,24 +684,24 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>Janeiro</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D14">
-        <v>539.15</v>
+        <v>520.3200000000001</v>
       </c>
       <c r="E14">
-        <v>3.9</v>
+        <v>-4.1</v>
       </c>
       <c r="F14" s="2">
         <v>45292</v>
@@ -710,24 +710,18 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>Fevereiro</t>
         </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
-      <c r="D15">
-        <v>540.36</v>
-      </c>
-      <c r="E15">
-        <v>0.23</v>
       </c>
       <c r="F15" s="2">
         <v>45323</v>
@@ -736,25 +730,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>Março</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
         </is>
       </c>
       <c r="D16">
         <v>514.03</v>
       </c>
-      <c r="E16">
-        <v>-4.87</v>
-      </c>
       <c r="F16" s="2">
         <v>45352</v>
       </c>
@@ -762,17 +753,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>Abril</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
         </is>
       </c>
       <c r="F17" s="2">
@@ -782,17 +773,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>Maio</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
         </is>
       </c>
       <c r="D18">
@@ -805,24 +796,24 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>Junho</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D19">
-        <v>628.8099999999999</v>
+        <v>610.36</v>
       </c>
       <c r="E19">
-        <v>4.34</v>
+        <v>1.27</v>
       </c>
       <c r="F19" s="2">
         <v>45444</v>
@@ -831,24 +822,24 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>Julho</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D20">
-        <v>610.4400000000001</v>
+        <v>563.7</v>
       </c>
       <c r="E20">
-        <v>-2.92</v>
+        <v>-7.64</v>
       </c>
       <c r="F20" s="2">
         <v>45474</v>
@@ -857,24 +848,24 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>Agosto</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
         </is>
       </c>
       <c r="D21">
         <v>538.58</v>
       </c>
       <c r="E21">
-        <v>-11.77</v>
+        <v>-4.46</v>
       </c>
       <c r="F21" s="2">
         <v>45505</v>
@@ -883,24 +874,24 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>Setembro</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D22">
-        <v>547.16</v>
+        <v>553.73</v>
       </c>
       <c r="E22">
-        <v>1.59</v>
+        <v>2.81</v>
       </c>
       <c r="F22" s="2">
         <v>45536</v>
@@ -909,24 +900,24 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>Outubro</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D23">
-        <v>553.84</v>
+        <v>558.39</v>
       </c>
       <c r="E23">
-        <v>1.22</v>
+        <v>0.84</v>
       </c>
       <c r="F23" s="2">
         <v>45566</v>
@@ -935,24 +926,24 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>Novembro</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D24">
-        <v>578.97</v>
+        <v>572.6900000000001</v>
       </c>
       <c r="E24">
-        <v>4.54</v>
+        <v>2.56</v>
       </c>
       <c r="F24" s="2">
         <v>45597</v>
@@ -961,24 +952,24 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>Dezembro</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D25">
-        <v>587.13</v>
+        <v>581.91</v>
       </c>
       <c r="E25">
-        <v>1.41</v>
+        <v>1.61</v>
       </c>
       <c r="F25" s="2">
         <v>45627</v>
@@ -987,24 +978,24 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Blumenau</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Janeiro</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Blumenau</t>
-        </is>
-      </c>
       <c r="D26">
-        <v>585.16</v>
+        <v>599.3099999999999</v>
       </c>
       <c r="E26">
-        <v>-0.34</v>
+        <v>2.99</v>
       </c>
       <c r="F26" s="2">
         <v>45658</v>
@@ -1013,330 +1004,474 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Janeiro</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Gaspar</t>
-        </is>
+          <t>Fevereiro</t>
+        </is>
+      </c>
+      <c r="D27">
+        <v>645.51</v>
+      </c>
+      <c r="E27">
+        <v>7.71</v>
       </c>
       <c r="F27" s="2">
-        <v>45292</v>
+        <v>45689</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="D28">
-        <v>596.15</v>
+        <v>665.86</v>
+      </c>
+      <c r="E28">
+        <v>3.15</v>
       </c>
       <c r="F28" s="2">
-        <v>45323</v>
+        <v>45717</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Blumenau</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Março</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gaspar</t>
-        </is>
-      </c>
-      <c r="D29">
-        <v>635.98</v>
-      </c>
-      <c r="E29">
-        <v>6.68</v>
+          <t>Abril</t>
+        </is>
       </c>
       <c r="F29" s="2">
-        <v>45352</v>
+        <v>45748</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Abril</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Gaspar</t>
-        </is>
-      </c>
-      <c r="D30">
-        <v>619.71</v>
-      </c>
-      <c r="E30">
-        <v>-2.56</v>
+          <t>Janeiro</t>
+        </is>
       </c>
       <c r="F30" s="2">
-        <v>45383</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Maio</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Fevereiro</t>
         </is>
       </c>
       <c r="D31">
-        <v>610.02</v>
-      </c>
-      <c r="E31">
-        <v>-1.56</v>
+        <v>596.15</v>
       </c>
       <c r="F31" s="2">
-        <v>45413</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Junho</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Março</t>
         </is>
       </c>
       <c r="D32">
-        <v>629.77</v>
+        <v>635.98</v>
       </c>
       <c r="E32">
-        <v>3.24</v>
+        <v>6.68</v>
       </c>
       <c r="F32" s="2">
-        <v>45444</v>
+        <v>45352</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Julho</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Abril</t>
         </is>
       </c>
       <c r="D33">
-        <v>581.67</v>
+        <v>619.71</v>
       </c>
       <c r="E33">
-        <v>-7.64</v>
+        <v>-2.56</v>
       </c>
       <c r="F33" s="2">
-        <v>45474</v>
+        <v>45383</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Agosto</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Maio</t>
         </is>
       </c>
       <c r="D34">
-        <v>580.99</v>
+        <v>610.02</v>
       </c>
       <c r="E34">
-        <v>-0.12</v>
+        <v>-1.56</v>
       </c>
       <c r="F34" s="2">
-        <v>45505</v>
+        <v>45413</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Setembro</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Junho</t>
         </is>
       </c>
       <c r="D35">
-        <v>588.79</v>
+        <v>629.77</v>
       </c>
       <c r="E35">
-        <v>1.34</v>
+        <v>3.24</v>
       </c>
       <c r="F35" s="2">
-        <v>45536</v>
+        <v>45444</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Outubro</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Julho</t>
         </is>
       </c>
       <c r="D36">
-        <v>554.67</v>
+        <v>581.67</v>
       </c>
       <c r="E36">
-        <v>-5.8</v>
+        <v>-7.64</v>
       </c>
       <c r="F36" s="2">
-        <v>45566</v>
+        <v>45474</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Novembro</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Agosto</t>
         </is>
       </c>
       <c r="D37">
-        <v>591.6</v>
+        <v>580.99</v>
       </c>
       <c r="E37">
-        <v>6.66</v>
+        <v>-0.12</v>
       </c>
       <c r="F37" s="2">
-        <v>45597</v>
+        <v>45505</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>Gaspar</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Dezembro</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Gaspar</t>
+          <t>Setembro</t>
         </is>
       </c>
       <c r="D38">
-        <v>565.35</v>
+        <v>588.79</v>
       </c>
       <c r="E38">
-        <v>-4.44</v>
+        <v>1.34</v>
       </c>
       <c r="F38" s="2">
-        <v>45627</v>
+        <v>45536</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>Gaspar</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Outubro</t>
+        </is>
+      </c>
+      <c r="D39">
+        <v>554.67</v>
+      </c>
+      <c r="E39">
+        <v>-5.8</v>
+      </c>
+      <c r="F39" s="2">
+        <v>45566</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Gaspar</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Novembro</t>
+        </is>
+      </c>
+      <c r="D40">
+        <v>591.6</v>
+      </c>
+      <c r="E40">
+        <v>6.66</v>
+      </c>
+      <c r="F40" s="2">
+        <v>45597</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Gaspar</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Dezembro</t>
+        </is>
+      </c>
+      <c r="D41">
+        <v>565.35</v>
+      </c>
+      <c r="E41">
+        <v>-4.44</v>
+      </c>
+      <c r="F41" s="2">
+        <v>45627</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Gaspar</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Janeiro</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Gaspar</t>
-        </is>
-      </c>
-      <c r="D39">
+      <c r="D42">
         <v>585.25</v>
       </c>
-      <c r="E39">
+      <c r="E42">
         <v>3.52</v>
       </c>
-      <c r="F39" s="2">
+      <c r="F42" s="2">
         <v>45658</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Gaspar</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Fevereiro</t>
+        </is>
+      </c>
+      <c r="D43">
+        <v>610.33</v>
+      </c>
+      <c r="E43">
+        <v>4.28</v>
+      </c>
+      <c r="F43" s="2">
+        <v>45689</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Gaspar</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Março</t>
+        </is>
+      </c>
+      <c r="D44">
+        <v>615.97</v>
+      </c>
+      <c r="E44">
+        <v>0.92</v>
+      </c>
+      <c r="F44" s="2">
+        <v>45717</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Gaspar</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Abril</t>
+        </is>
+      </c>
+      <c r="F45" s="2">
+        <v>45748</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ok, corrected Outubro 2023
</commit_message>
<xml_diff>
--- a/CT.xlsx
+++ b/CT.xlsx
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="D5">
-        <v>530.74</v>
+        <v>531.49</v>
       </c>
       <c r="E5">
-        <v>-0.7</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="F5" s="2">
         <v>45017</v>
@@ -542,10 +542,10 @@
         </is>
       </c>
       <c r="D8">
-        <v>547.9400000000001</v>
+        <v>532.25</v>
       </c>
       <c r="E8">
-        <v>-2.2</v>
+        <v>-5</v>
       </c>
       <c r="F8" s="2">
         <v>45108</v>
@@ -568,10 +568,10 @@
         </is>
       </c>
       <c r="D9">
-        <v>528.54</v>
+        <v>523.8</v>
       </c>
       <c r="E9">
-        <v>-3.54</v>
+        <v>-1.59</v>
       </c>
       <c r="F9" s="2">
         <v>45139</v>
@@ -594,10 +594,10 @@
         </is>
       </c>
       <c r="D10">
-        <v>514.08</v>
+        <v>516.0599999999999</v>
       </c>
       <c r="E10">
-        <v>-2.74</v>
+        <v>-1.48</v>
       </c>
       <c r="F10" s="2">
         <v>45170</v>
@@ -619,12 +619,6 @@
           <t>Outubro</t>
         </is>
       </c>
-      <c r="D11">
-        <v>806.37</v>
-      </c>
-      <c r="E11">
-        <v>56.86</v>
-      </c>
       <c r="F11" s="2">
         <v>45200</v>
       </c>
@@ -648,9 +642,6 @@
       <c r="D12">
         <v>547.5700000000001</v>
       </c>
-      <c r="E12">
-        <v>-32.09</v>
-      </c>
       <c r="F12" s="2">
         <v>45231</v>
       </c>
@@ -672,10 +663,10 @@
         </is>
       </c>
       <c r="D13">
-        <v>542.55</v>
+        <v>515.79</v>
       </c>
       <c r="E13">
-        <v>-0.92</v>
+        <v>-5.8</v>
       </c>
       <c r="F13" s="2">
         <v>45261</v>
@@ -701,7 +692,7 @@
         <v>520.3200000000001</v>
       </c>
       <c r="E14">
-        <v>-4.1</v>
+        <v>0.88</v>
       </c>
       <c r="F14" s="2">
         <v>45292</v>

</xml_diff>